<commit_message>
Add backlog, prod, and saida_sem_it - 2026-09-23 18:30:03
</commit_message>
<xml_diff>
--- a/SaidaSemITGATEAutoCompleto.xlsx
+++ b/SaidaSemITGATEAutoCompleto.xlsx
@@ -40679,16 +40679,16 @@
         <v>1606</v>
       </c>
       <c r="C770" t="s">
-        <v>2015</v>
+        <v>1910</v>
       </c>
       <c r="D770" t="s">
-        <v>2033</v>
+        <v>1910</v>
       </c>
       <c r="E770" t="s">
-        <v>2033</v>
+        <v>1910</v>
       </c>
       <c r="F770" s="2">
-        <v>46286</v>
+        <v>46288</v>
       </c>
       <c r="G770" t="s">
         <v>2106</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-10-16 12:30:04
</commit_message>
<xml_diff>
--- a/SaidaSemITGATEAutoCompleto.xlsx
+++ b/SaidaSemITGATEAutoCompleto.xlsx
@@ -30227,10 +30227,10 @@
         <v>1301</v>
       </c>
       <c r="C445" t="s">
-        <v>1932</v>
+        <v>1755</v>
       </c>
       <c r="F445" s="2">
-        <v>46185</v>
+        <v>46311</v>
       </c>
       <c r="G445" t="s">
         <v>2159</v>
@@ -39009,10 +39009,10 @@
         <v>1564</v>
       </c>
       <c r="C708" t="s">
-        <v>1976</v>
+        <v>1826</v>
       </c>
       <c r="F708" s="2">
-        <v>45994</v>
+        <v>46311</v>
       </c>
       <c r="G708" t="s">
         <v>2159</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-10-27 10:30:03
</commit_message>
<xml_diff>
--- a/SaidaSemITGATEAutoCompleto.xlsx
+++ b/SaidaSemITGATEAutoCompleto.xlsx
@@ -6205,177 +6205,180 @@
     <t>12/08/2025</t>
   </si>
   <si>
+    <t>05/08/2026</t>
+  </si>
+  <si>
+    <t>04/11/2024</t>
+  </si>
+  <si>
+    <t>17/07/2025</t>
+  </si>
+  <si>
+    <t>09/07/2025</t>
+  </si>
+  <si>
+    <t>27/11/2025</t>
+  </si>
+  <si>
+    <t>23/09/2026</t>
+  </si>
+  <si>
+    <t>19/03/2025</t>
+  </si>
+  <si>
+    <t>14/07/2026</t>
+  </si>
+  <si>
+    <t>09/06/2026</t>
+  </si>
+  <si>
+    <t>13/10/2025</t>
+  </si>
+  <si>
+    <t>10/06/2025</t>
+  </si>
+  <si>
+    <t>10/07/2025</t>
+  </si>
+  <si>
+    <t>28/02/2025</t>
+  </si>
+  <si>
+    <t>19/11/2024</t>
+  </si>
+  <si>
+    <t>23/01/2025</t>
+  </si>
+  <si>
+    <t>25/09/2025</t>
+  </si>
+  <si>
+    <t>26/07/2024</t>
+  </si>
+  <si>
+    <t>10/04/2026</t>
+  </si>
+  <si>
+    <t>15/07/2026</t>
+  </si>
+  <si>
+    <t>15/05/2026</t>
+  </si>
+  <si>
+    <t>25/09/2026</t>
+  </si>
+  <si>
+    <t>07/10/2026</t>
+  </si>
+  <si>
+    <t>09/10/2025</t>
+  </si>
+  <si>
+    <t>22/01/2025</t>
+  </si>
+  <si>
+    <t>13/06/2025</t>
+  </si>
+  <si>
+    <t>02/06/2026</t>
+  </si>
+  <si>
+    <t>08/10/2025</t>
+  </si>
+  <si>
+    <t>06/02/2025</t>
+  </si>
+  <si>
+    <t>01/08/2025</t>
+  </si>
+  <si>
+    <t>19/02/2025</t>
+  </si>
+  <si>
+    <t>03/12/2025</t>
+  </si>
+  <si>
+    <t>11/03/2026</t>
+  </si>
+  <si>
+    <t>24/08/2026</t>
+  </si>
+  <si>
+    <t>16/02/2024</t>
+  </si>
+  <si>
+    <t>29/03/2022</t>
+  </si>
+  <si>
+    <t>28/04/2025</t>
+  </si>
+  <si>
+    <t>21/11/2024</t>
+  </si>
+  <si>
+    <t>27/02/2025</t>
+  </si>
+  <si>
+    <t>06/11/2025</t>
+  </si>
+  <si>
+    <t>05/06/2025</t>
+  </si>
+  <si>
+    <t>28/01/2026</t>
+  </si>
+  <si>
+    <t>10/08/2026</t>
+  </si>
+  <si>
+    <t>02/10/2024</t>
+  </si>
+  <si>
+    <t>05/08/2024</t>
+  </si>
+  <si>
+    <t>13/11/2025</t>
+  </si>
+  <si>
+    <t>24/09/2026</t>
+  </si>
+  <si>
+    <t>04/09/2025</t>
+  </si>
+  <si>
+    <t>20/11/2025</t>
+  </si>
+  <si>
+    <t>12/11/2025</t>
+  </si>
+  <si>
+    <t>03/01/2025</t>
+  </si>
+  <si>
+    <t>13/09/2024</t>
+  </si>
+  <si>
+    <t>29/09/2026</t>
+  </si>
+  <si>
+    <t>26/08/2026</t>
+  </si>
+  <si>
+    <t>22/01/2026</t>
+  </si>
+  <si>
+    <t>04/07/2025</t>
+  </si>
+  <si>
+    <t>31/07/2025</t>
+  </si>
+  <si>
+    <t>07/07/2026</t>
+  </si>
+  <si>
     <t>13/03/2026</t>
   </si>
   <si>
-    <t>04/11/2024</t>
-  </si>
-  <si>
-    <t>17/07/2025</t>
-  </si>
-  <si>
-    <t>09/07/2025</t>
-  </si>
-  <si>
-    <t>27/11/2025</t>
-  </si>
-  <si>
-    <t>23/09/2026</t>
-  </si>
-  <si>
-    <t>19/03/2025</t>
-  </si>
-  <si>
-    <t>14/07/2026</t>
-  </si>
-  <si>
-    <t>09/06/2026</t>
-  </si>
-  <si>
-    <t>13/10/2025</t>
-  </si>
-  <si>
-    <t>10/06/2025</t>
-  </si>
-  <si>
-    <t>10/07/2025</t>
-  </si>
-  <si>
-    <t>28/02/2025</t>
-  </si>
-  <si>
-    <t>19/11/2024</t>
-  </si>
-  <si>
-    <t>23/01/2025</t>
-  </si>
-  <si>
-    <t>25/09/2025</t>
-  </si>
-  <si>
-    <t>26/07/2024</t>
-  </si>
-  <si>
-    <t>10/04/2026</t>
-  </si>
-  <si>
-    <t>15/07/2026</t>
-  </si>
-  <si>
-    <t>15/05/2026</t>
-  </si>
-  <si>
-    <t>25/09/2026</t>
-  </si>
-  <si>
-    <t>07/10/2026</t>
-  </si>
-  <si>
-    <t>09/10/2025</t>
-  </si>
-  <si>
-    <t>22/01/2025</t>
-  </si>
-  <si>
-    <t>13/06/2025</t>
-  </si>
-  <si>
-    <t>02/06/2026</t>
-  </si>
-  <si>
-    <t>08/10/2025</t>
-  </si>
-  <si>
-    <t>06/02/2025</t>
-  </si>
-  <si>
-    <t>01/08/2025</t>
-  </si>
-  <si>
-    <t>19/02/2025</t>
-  </si>
-  <si>
-    <t>03/12/2025</t>
-  </si>
-  <si>
-    <t>11/03/2026</t>
-  </si>
-  <si>
-    <t>24/08/2026</t>
-  </si>
-  <si>
-    <t>16/02/2024</t>
-  </si>
-  <si>
-    <t>29/03/2022</t>
-  </si>
-  <si>
-    <t>28/04/2025</t>
-  </si>
-  <si>
-    <t>21/11/2024</t>
-  </si>
-  <si>
-    <t>27/02/2025</t>
-  </si>
-  <si>
-    <t>06/11/2025</t>
-  </si>
-  <si>
-    <t>05/06/2025</t>
-  </si>
-  <si>
-    <t>28/01/2026</t>
-  </si>
-  <si>
-    <t>10/08/2026</t>
-  </si>
-  <si>
-    <t>02/10/2024</t>
-  </si>
-  <si>
-    <t>05/08/2024</t>
-  </si>
-  <si>
-    <t>13/11/2025</t>
-  </si>
-  <si>
-    <t>24/09/2026</t>
-  </si>
-  <si>
-    <t>04/09/2025</t>
-  </si>
-  <si>
-    <t>20/11/2025</t>
-  </si>
-  <si>
-    <t>12/11/2025</t>
-  </si>
-  <si>
-    <t>03/01/2025</t>
-  </si>
-  <si>
-    <t>13/09/2024</t>
-  </si>
-  <si>
-    <t>29/09/2026</t>
-  </si>
-  <si>
-    <t>26/08/2026</t>
-  </si>
-  <si>
-    <t>22/01/2026</t>
-  </si>
-  <si>
-    <t>04/07/2025</t>
-  </si>
-  <si>
-    <t>31/07/2025</t>
-  </si>
-  <si>
-    <t>07/07/2026</t>
-  </si>
-  <si>
     <t>08/05/2026</t>
   </si>
   <si>
@@ -6434,9 +6437,6 @@
   </si>
   <si>
     <t>26/05/2026</t>
-  </si>
-  <si>
-    <t>05/08/2026</t>
   </si>
   <si>
     <t>19/09/2024</t>
@@ -15726,10 +15726,10 @@
         <v>1730</v>
       </c>
       <c r="D4" t="s">
-        <v>2122</v>
+        <v>2123</v>
       </c>
       <c r="E4" t="s">
-        <v>2122</v>
+        <v>2123</v>
       </c>
       <c r="F4" s="2">
         <v>45709</v>
@@ -15764,10 +15764,10 @@
         <v>1731</v>
       </c>
       <c r="D5" t="s">
-        <v>2123</v>
+        <v>2124</v>
       </c>
       <c r="E5" t="s">
-        <v>2123</v>
+        <v>2124</v>
       </c>
       <c r="F5" s="2">
         <v>46260</v>
@@ -15805,7 +15805,7 @@
         <v>1847</v>
       </c>
       <c r="E6" t="s">
-        <v>2140</v>
+        <v>2063</v>
       </c>
       <c r="F6" s="2">
         <v>46274</v>
@@ -16032,7 +16032,7 @@
         <v>1739</v>
       </c>
       <c r="D13" t="s">
-        <v>2124</v>
+        <v>2125</v>
       </c>
       <c r="E13" t="s">
         <v>2062</v>
@@ -16198,10 +16198,10 @@
         <v>1744</v>
       </c>
       <c r="D18" t="s">
-        <v>2120</v>
+        <v>2121</v>
       </c>
       <c r="E18" t="s">
-        <v>2137</v>
+        <v>2138</v>
       </c>
       <c r="F18" s="2">
         <v>46247</v>
@@ -16428,10 +16428,10 @@
         <v>1750</v>
       </c>
       <c r="D25" t="s">
-        <v>2125</v>
+        <v>2126</v>
       </c>
       <c r="E25" t="s">
-        <v>2125</v>
+        <v>2126</v>
       </c>
       <c r="F25" s="2">
         <v>46183</v>
@@ -16967,7 +16967,7 @@
         <v>1765</v>
       </c>
       <c r="D41" t="s">
-        <v>2126</v>
+        <v>2127</v>
       </c>
       <c r="F41" s="2">
         <v>46090</v>
@@ -18288,7 +18288,7 @@
         <v>1804</v>
       </c>
       <c r="D82" t="s">
-        <v>2127</v>
+        <v>2128</v>
       </c>
       <c r="E82" t="s">
         <v>2067</v>
@@ -18390,10 +18390,10 @@
         <v>1807</v>
       </c>
       <c r="D85" t="s">
-        <v>2128</v>
+        <v>2129</v>
       </c>
       <c r="E85" t="s">
-        <v>2128</v>
+        <v>2129</v>
       </c>
       <c r="F85" s="2">
         <v>45846</v>
@@ -18428,10 +18428,10 @@
         <v>1808</v>
       </c>
       <c r="D86" t="s">
-        <v>2125</v>
+        <v>2126</v>
       </c>
       <c r="E86" t="s">
-        <v>2125</v>
+        <v>2126</v>
       </c>
       <c r="F86" s="2">
         <v>46182</v>
@@ -18562,7 +18562,7 @@
         <v>1811</v>
       </c>
       <c r="D90" t="s">
-        <v>2129</v>
+        <v>2130</v>
       </c>
       <c r="E90" t="s">
         <v>2175</v>
@@ -19229,7 +19229,7 @@
         <v>1825</v>
       </c>
       <c r="D110" t="s">
-        <v>2130</v>
+        <v>2131</v>
       </c>
       <c r="F110" s="2">
         <v>46111</v>
@@ -19785,10 +19785,10 @@
         <v>1811</v>
       </c>
       <c r="D127" t="s">
-        <v>2131</v>
+        <v>2132</v>
       </c>
       <c r="E127" t="s">
-        <v>2131</v>
+        <v>2132</v>
       </c>
       <c r="F127" s="2">
         <v>46079</v>
@@ -19995,7 +19995,7 @@
         <v>1841</v>
       </c>
       <c r="D133" t="s">
-        <v>2132</v>
+        <v>2133</v>
       </c>
       <c r="E133" t="s">
         <v>1932</v>
@@ -20196,10 +20196,10 @@
         <v>1828</v>
       </c>
       <c r="D139" t="s">
-        <v>2133</v>
+        <v>2134</v>
       </c>
       <c r="E139" t="s">
-        <v>2133</v>
+        <v>2134</v>
       </c>
       <c r="F139" s="2">
         <v>46184</v>
@@ -20607,10 +20607,10 @@
         <v>1768</v>
       </c>
       <c r="D151" t="s">
-        <v>2125</v>
+        <v>2126</v>
       </c>
       <c r="E151" t="s">
-        <v>2125</v>
+        <v>2126</v>
       </c>
       <c r="F151" s="2">
         <v>46175</v>
@@ -20744,7 +20744,7 @@
         <v>1854</v>
       </c>
       <c r="D155" t="s">
-        <v>2134</v>
+        <v>2135</v>
       </c>
       <c r="E155" t="s">
         <v>1980</v>
@@ -20945,7 +20945,7 @@
         <v>1859</v>
       </c>
       <c r="D161" t="s">
-        <v>2135</v>
+        <v>2136</v>
       </c>
       <c r="F161" s="2">
         <v>45804</v>
@@ -21181,7 +21181,7 @@
         <v>1730</v>
       </c>
       <c r="D168" t="s">
-        <v>2136</v>
+        <v>2137</v>
       </c>
       <c r="E168" t="s">
         <v>1948</v>
@@ -21481,10 +21481,10 @@
         <v>1866</v>
       </c>
       <c r="D177" t="s">
-        <v>2137</v>
+        <v>2138</v>
       </c>
       <c r="E177" t="s">
-        <v>2137</v>
+        <v>2138</v>
       </c>
       <c r="F177" s="2">
         <v>46148</v>
@@ -22227,10 +22227,10 @@
         <v>1882</v>
       </c>
       <c r="D199" t="s">
-        <v>2138</v>
+        <v>2139</v>
       </c>
       <c r="E199" t="s">
-        <v>2138</v>
+        <v>2139</v>
       </c>
       <c r="F199" s="2">
         <v>45684</v>
@@ -22367,7 +22367,7 @@
         <v>1762</v>
       </c>
       <c r="D203" t="s">
-        <v>2139</v>
+        <v>2140</v>
       </c>
       <c r="E203" t="s">
         <v>1818</v>
@@ -23156,7 +23156,7 @@
         <v>2096</v>
       </c>
       <c r="E227" t="s">
-        <v>2121</v>
+        <v>2122</v>
       </c>
       <c r="F227" s="2">
         <v>45876</v>
@@ -23587,7 +23587,7 @@
         <v>1774</v>
       </c>
       <c r="E240" t="s">
-        <v>2121</v>
+        <v>2122</v>
       </c>
       <c r="F240" s="2">
         <v>45894</v>
@@ -23963,10 +23963,10 @@
         <v>1823</v>
       </c>
       <c r="D251" t="s">
-        <v>2140</v>
+        <v>2063</v>
       </c>
       <c r="E251" t="s">
-        <v>2140</v>
+        <v>2063</v>
       </c>
       <c r="F251" s="2">
         <v>46246</v>
@@ -27069,10 +27069,10 @@
         <v>1897</v>
       </c>
       <c r="D343" t="s">
-        <v>2133</v>
+        <v>2134</v>
       </c>
       <c r="E343" t="s">
-        <v>2133</v>
+        <v>2134</v>
       </c>
       <c r="F343" s="2">
         <v>46112</v>
@@ -27538,10 +27538,10 @@
         <v>1971</v>
       </c>
       <c r="D357" t="s">
-        <v>2137</v>
+        <v>2138</v>
       </c>
       <c r="E357" t="s">
-        <v>2137</v>
+        <v>2138</v>
       </c>
       <c r="F357" s="2">
         <v>46157</v>
@@ -28182,10 +28182,10 @@
         <v>1980</v>
       </c>
       <c r="D376" t="s">
-        <v>2137</v>
+        <v>2138</v>
       </c>
       <c r="E376" t="s">
-        <v>2137</v>
+        <v>2138</v>
       </c>
       <c r="F376" s="2">
         <v>46232</v>
@@ -28884,7 +28884,7 @@
         <v>2004</v>
       </c>
       <c r="E397" t="s">
-        <v>2131</v>
+        <v>2132</v>
       </c>
       <c r="F397" s="2">
         <v>46254</v>
@@ -30081,7 +30081,7 @@
         <v>1729</v>
       </c>
       <c r="E433" t="s">
-        <v>2125</v>
+        <v>2126</v>
       </c>
       <c r="F433" s="2">
         <v>46170</v>
@@ -33858,10 +33858,10 @@
         <v>2017</v>
       </c>
       <c r="D547" t="s">
-        <v>2125</v>
+        <v>2126</v>
       </c>
       <c r="E547" t="s">
-        <v>2125</v>
+        <v>2126</v>
       </c>
       <c r="F547" s="2">
         <v>46176</v>
@@ -35355,10 +35355,10 @@
         <v>2061</v>
       </c>
       <c r="D592" t="s">
-        <v>2125</v>
+        <v>2126</v>
       </c>
       <c r="E592" t="s">
-        <v>2125</v>
+        <v>2126</v>
       </c>
       <c r="F592" s="2">
         <v>46175</v>
@@ -35556,7 +35556,7 @@
         <v>2063</v>
       </c>
       <c r="F598" s="2">
-        <v>46188</v>
+        <v>46322</v>
       </c>
       <c r="G598" t="s">
         <v>2188</v>
@@ -39364,7 +39364,7 @@
         <v>2088</v>
       </c>
       <c r="E711" t="s">
-        <v>2137</v>
+        <v>2138</v>
       </c>
       <c r="F711" s="2">
         <v>46176</v>
@@ -39909,7 +39909,7 @@
         <v>2093</v>
       </c>
       <c r="D727" t="s">
-        <v>2129</v>
+        <v>2130</v>
       </c>
       <c r="E727" t="s">
         <v>2187</v>
@@ -40978,7 +40978,7 @@
         <v>1802</v>
       </c>
       <c r="E759" t="s">
-        <v>2121</v>
+        <v>2122</v>
       </c>
       <c r="F759" s="2">
         <v>45799</v>
@@ -41179,10 +41179,10 @@
         <v>1771</v>
       </c>
       <c r="D765" t="s">
-        <v>2131</v>
+        <v>2132</v>
       </c>
       <c r="E765" t="s">
-        <v>2131</v>
+        <v>2132</v>
       </c>
       <c r="F765" s="2">
         <v>46091</v>
@@ -42953,10 +42953,10 @@
         <v>2015</v>
       </c>
       <c r="D818" t="s">
-        <v>2137</v>
+        <v>2138</v>
       </c>
       <c r="E818" t="s">
-        <v>2137</v>
+        <v>2138</v>
       </c>
       <c r="F818" s="2">
         <v>46167</v>
@@ -43891,7 +43891,7 @@
         <v>1714</v>
       </c>
       <c r="C846" t="s">
-        <v>2063</v>
+        <v>2120</v>
       </c>
       <c r="D846" t="s">
         <v>1742</v>
@@ -43929,7 +43929,7 @@
         <v>1715</v>
       </c>
       <c r="C847" t="s">
-        <v>2120</v>
+        <v>2121</v>
       </c>
       <c r="F847" s="2">
         <v>46258</v>
@@ -44229,7 +44229,7 @@
         <v>1724</v>
       </c>
       <c r="C856" t="s">
-        <v>2121</v>
+        <v>2122</v>
       </c>
       <c r="F856" s="2">
         <v>45762</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-10-28 10:30:04
</commit_message>
<xml_diff>
--- a/SaidaSemITGATEAutoCompleto.xlsx
+++ b/SaidaSemITGATEAutoCompleto.xlsx
@@ -35722,10 +35722,10 @@
         <v>1471</v>
       </c>
       <c r="C603" t="s">
-        <v>1946</v>
+        <v>1911</v>
       </c>
       <c r="F603" s="2">
-        <v>45946</v>
+        <v>46323</v>
       </c>
       <c r="G603" t="s">
         <v>2189</v>

</xml_diff>